<commit_message>
Smaller irl accurate model, x,y,z box coordinates replaced by discretisized space in the container based on the input set of pallets and their dimensions
</commit_message>
<xml_diff>
--- a/sample_instances/input_small.xlsx
+++ b/sample_instances/input_small.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="76">
   <si>
     <t>Barcode Item</t>
   </si>
@@ -224,9 +224,6 @@
   </si>
   <si>
     <t>1.15x1.15x1.22</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Blockpallet 1.15x1.15x1.22m  8 sets</t>
@@ -271,7 +268,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -396,7 +393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="30">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -458,15 +455,6 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -480,13 +468,13 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -799,32 +787,32 @@
   <dimension ref="A1:W36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="28" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="29" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="30" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="4" max="4" style="30" width="58.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="30" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="6" max="6" style="30" width="26.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="30" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="8" max="8" style="31" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="9" max="9" style="31" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="10" max="10" style="32" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="11" max="11" style="29" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="31" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="13" max="13" style="30" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="14" max="14" style="30" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="15" max="15" style="30" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="16" max="16" style="32" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="17" max="17" style="29" width="22.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="29" width="19.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="30" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="20" max="20" style="31" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="21" max="21" style="31" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="22" max="22" style="31" width="12.43357142857143" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="23" max="23" style="30" width="8.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="25" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="26" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="27" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="4" max="4" style="27" width="58.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="27" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="6" max="6" style="27" width="26.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="27" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="8" max="8" style="28" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="9" max="9" style="28" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="10" max="10" style="29" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="11" max="11" style="26" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="28" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="13" max="13" style="27" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="14" max="14" style="27" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="15" max="15" style="27" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="16" max="16" style="29" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="17" max="17" style="26" width="22.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="26" width="19.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="27" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="20" max="20" style="28" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="21" max="21" style="28" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="22" max="22" style="28" width="13.005" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="23" max="23" style="27" width="8.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -863,7 +851,7 @@
       <c r="V1" s="7"/>
       <c r="W1" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="12" t="s">
         <v>7</v>
       </c>
@@ -891,7 +879,7 @@
       <c r="O2" s="6"/>
       <c r="P2" s="8"/>
       <c r="Q2" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R2" s="15">
         <v>12</v>
@@ -902,7 +890,7 @@
       <c r="V2" s="7"/>
       <c r="W2" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="12" t="s">
         <v>10</v>
       </c>
@@ -952,7 +940,7 @@
         <v>23</v>
       </c>
       <c r="Q3" s="7">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="R3" s="15">
         <v>9</v>
@@ -969,7 +957,7 @@
       </c>
       <c r="W3" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="12" t="s">
         <v>27</v>
       </c>
@@ -1036,7 +1024,7 @@
       </c>
       <c r="W4" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="12" t="s">
         <v>36</v>
       </c>
@@ -1103,7 +1091,7 @@
       </c>
       <c r="W5" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="12" t="s">
         <v>40</v>
       </c>
@@ -1170,7 +1158,7 @@
       </c>
       <c r="W6" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="12" t="s">
         <v>44</v>
       </c>
@@ -1237,7 +1225,7 @@
       </c>
       <c r="W7" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="12" t="s">
         <v>47</v>
       </c>
@@ -1304,7 +1292,7 @@
       </c>
       <c r="W8" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="12" t="s">
         <v>51</v>
       </c>
@@ -1371,7 +1359,7 @@
       </c>
       <c r="W9" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="12" t="s">
         <v>53</v>
       </c>
@@ -1438,7 +1426,7 @@
       </c>
       <c r="W10" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="12" t="s">
         <v>56</v>
       </c>
@@ -1505,7 +1493,7 @@
       </c>
       <c r="W11" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="12" t="s">
         <v>58</v>
       </c>
@@ -1553,7 +1541,7 @@
         <v>118.32</v>
       </c>
       <c r="Q12" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R12" s="15">
         <v>5</v>
@@ -1572,7 +1560,7 @@
       </c>
       <c r="W12" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="12" t="s">
         <v>60</v>
       </c>
@@ -1620,7 +1608,7 @@
         <v>167</v>
       </c>
       <c r="Q13" s="7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R13" s="15">
         <v>24</v>
@@ -1639,7 +1627,7 @@
       </c>
       <c r="W13" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="12" t="s">
         <v>62</v>
       </c>
@@ -1687,7 +1675,7 @@
         <v>167</v>
       </c>
       <c r="Q14" s="7">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="R14" s="15">
         <v>15</v>
@@ -1706,7 +1694,7 @@
       </c>
       <c r="W14" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="12" t="s">
         <v>64</v>
       </c>
@@ -1754,7 +1742,7 @@
         <v>103.37</v>
       </c>
       <c r="Q15" s="7">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="R15" s="15">
         <v>5</v>
@@ -1773,7 +1761,7 @@
       </c>
       <c r="W15" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="12" t="s">
         <v>66</v>
       </c>
@@ -1821,7 +1809,7 @@
         <v>153.22</v>
       </c>
       <c r="Q16" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R16" s="15">
         <v>40</v>
@@ -1840,21 +1828,15 @@
       </c>
       <c r="W16" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
-      <c r="A17" s="21" t="s">
-        <v>69</v>
-      </c>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="21"/>
       <c r="B17" s="13"/>
       <c r="C17" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D17" s="3"/>
       <c r="E17" s="3"/>
-      <c r="F17" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F17" s="14"/>
       <c r="G17" s="6" t="s">
         <v>50</v>
       </c>
@@ -1899,23 +1881,17 @@
       </c>
       <c r="W17" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
-      <c r="A18" s="21" t="s">
-        <v>69</v>
-      </c>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="21"/>
       <c r="B18" s="13"/>
       <c r="C18" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="E18" s="3"/>
-      <c r="F18" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="H18" s="7">
         <v>40</v>
@@ -1958,23 +1934,17 @@
       </c>
       <c r="W18" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
-      <c r="A19" s="21" t="s">
-        <v>69</v>
-      </c>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+      <c r="A19" s="21"/>
       <c r="B19" s="13"/>
       <c r="C19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D19" s="3"/>
       <c r="E19" s="3"/>
-      <c r="F19" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F19" s="14"/>
       <c r="G19" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H19" s="7">
         <v>44</v>
@@ -2017,23 +1987,17 @@
       </c>
       <c r="W19" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
-      <c r="A20" s="21" t="s">
-        <v>69</v>
-      </c>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="A20" s="21"/>
       <c r="B20" s="13"/>
       <c r="C20" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D20" s="3"/>
       <c r="E20" s="3"/>
-      <c r="F20" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F20" s="14"/>
       <c r="G20" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H20" s="7">
         <v>90</v>
@@ -2076,23 +2040,17 @@
       </c>
       <c r="W20" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
-      <c r="A21" s="21" t="s">
-        <v>69</v>
-      </c>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="A21" s="21"/>
       <c r="B21" s="13"/>
       <c r="C21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="E21" s="3"/>
-      <c r="F21" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="H21" s="7">
         <v>40</v>
@@ -2135,23 +2093,17 @@
       </c>
       <c r="W21" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
-      <c r="A22" s="21" t="s">
-        <v>69</v>
-      </c>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="A22" s="21"/>
       <c r="B22" s="13"/>
       <c r="C22" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D22" s="3"/>
       <c r="E22" s="3"/>
-      <c r="F22" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F22" s="14"/>
       <c r="G22" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H22" s="7">
         <v>44</v>
@@ -2194,23 +2146,17 @@
       </c>
       <c r="W22" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
-      <c r="A23" s="21" t="s">
-        <v>69</v>
-      </c>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="A23" s="21"/>
       <c r="B23" s="13"/>
       <c r="C23" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D23" s="3"/>
       <c r="E23" s="3"/>
-      <c r="F23" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F23" s="14"/>
       <c r="G23" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H23" s="7">
         <v>90</v>
@@ -2254,22 +2200,16 @@
       <c r="W23" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
-      <c r="A24" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A24" s="21"/>
       <c r="B24" s="13"/>
       <c r="C24" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="E24" s="3"/>
-      <c r="F24" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="H24" s="7">
         <v>40</v>
@@ -2313,22 +2253,16 @@
       <c r="W24" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
-      <c r="A25" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A25" s="21"/>
       <c r="B25" s="13"/>
       <c r="C25" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D25" s="3"/>
       <c r="E25" s="3"/>
-      <c r="F25" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F25" s="14"/>
       <c r="G25" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H25" s="7">
         <v>44</v>
@@ -2372,22 +2306,16 @@
       <c r="W25" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
-      <c r="A26" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A26" s="21"/>
       <c r="B26" s="13"/>
       <c r="C26" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D26" s="3"/>
       <c r="E26" s="3"/>
-      <c r="F26" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F26" s="14"/>
       <c r="G26" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H26" s="7">
         <v>90</v>
@@ -2431,22 +2359,16 @@
       <c r="W26" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25">
-      <c r="A27" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A27" s="21"/>
       <c r="B27" s="13"/>
       <c r="C27" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D27" s="3"/>
       <c r="E27" s="3"/>
-      <c r="F27" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F27" s="14"/>
       <c r="G27" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H27" s="7">
         <v>88</v>
@@ -2490,22 +2412,16 @@
       <c r="W27" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="17.25">
-      <c r="A28" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A28" s="21"/>
       <c r="B28" s="13"/>
       <c r="C28" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D28" s="3"/>
       <c r="E28" s="3"/>
-      <c r="F28" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F28" s="14"/>
       <c r="G28" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H28" s="7">
         <v>88</v>
@@ -2549,22 +2465,16 @@
       <c r="W28" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="17.25">
-      <c r="A29" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A29" s="21"/>
       <c r="B29" s="13"/>
       <c r="C29" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D29" s="3"/>
       <c r="E29" s="3"/>
-      <c r="F29" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F29" s="14"/>
       <c r="G29" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H29" s="7">
         <v>88</v>
@@ -2608,22 +2518,16 @@
       <c r="W29" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25">
-      <c r="A30" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A30" s="21"/>
       <c r="B30" s="13"/>
       <c r="C30" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D30" s="22" t="s">
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="E30" s="3"/>
-      <c r="F30" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="H30" s="7">
         <v>40</v>
@@ -2667,22 +2571,16 @@
       <c r="W30" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
-      <c r="A31" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A31" s="21"/>
       <c r="B31" s="13"/>
       <c r="C31" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D31" s="3"/>
       <c r="E31" s="3"/>
-      <c r="F31" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F31" s="14"/>
       <c r="G31" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H31" s="7">
         <v>44</v>
@@ -2726,22 +2624,16 @@
       <c r="W31" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25">
-      <c r="A32" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A32" s="21"/>
       <c r="B32" s="13"/>
       <c r="C32" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D32" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D32" s="3"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F32" s="14"/>
       <c r="G32" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H32" s="7">
         <v>90</v>
@@ -2785,22 +2677,16 @@
       <c r="W32" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25">
-      <c r="A33" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A33" s="21"/>
       <c r="B33" s="13"/>
       <c r="C33" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D33" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D33" s="3"/>
       <c r="E33" s="3"/>
-      <c r="F33" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F33" s="14"/>
       <c r="G33" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H33" s="7">
         <v>80</v>
@@ -2844,22 +2730,16 @@
       <c r="W33" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="17.25">
-      <c r="A34" s="21" t="s">
-        <v>69</v>
-      </c>
+      <c r="A34" s="21"/>
       <c r="B34" s="13"/>
       <c r="C34" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D34" s="22" t="s">
-        <v>69</v>
-      </c>
+      <c r="D34" s="3"/>
       <c r="E34" s="3"/>
-      <c r="F34" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F34" s="14"/>
       <c r="G34" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H34" s="7">
         <v>80</v>
@@ -2903,8 +2783,8 @@
       <c r="W34" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="17.25">
-      <c r="A35" s="12"/>
-      <c r="B35" s="24"/>
+      <c r="A35" s="21"/>
+      <c r="B35" s="21"/>
       <c r="C35" s="3" t="s">
         <v>28</v>
       </c>
@@ -2912,7 +2792,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H35" s="13">
         <v>80</v>
@@ -2920,10 +2800,10 @@
       <c r="I35" s="13">
         <v>400</v>
       </c>
-      <c r="J35" s="25">
+      <c r="J35" s="22">
         <v>0.80624436</v>
       </c>
-      <c r="K35" s="26"/>
+      <c r="K35" s="23"/>
       <c r="L35" s="13">
         <v>0</v>
       </c>
@@ -2936,28 +2816,28 @@
       <c r="O35" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="P35" s="25">
+      <c r="P35" s="22">
         <v>69.35</v>
       </c>
-      <c r="Q35" s="24"/>
-      <c r="R35" s="26"/>
+      <c r="Q35" s="21"/>
+      <c r="R35" s="23"/>
       <c r="S35" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="T35" s="25">
+      <c r="T35" s="22">
         <v>346.75</v>
       </c>
-      <c r="U35" s="25">
+      <c r="U35" s="22">
         <v>0.80624436</v>
       </c>
-      <c r="V35" s="25">
+      <c r="V35" s="22">
         <v>0.0139007648275862</v>
       </c>
-      <c r="W35" s="27"/>
+      <c r="W35" s="24"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="17.25">
-      <c r="A36" s="12"/>
-      <c r="B36" s="24"/>
+      <c r="A36" s="21"/>
+      <c r="B36" s="21"/>
       <c r="C36" s="3" t="s">
         <v>28</v>
       </c>
@@ -2965,7 +2845,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H36" s="13">
         <v>60</v>
@@ -2973,10 +2853,10 @@
       <c r="I36" s="13">
         <v>720</v>
       </c>
-      <c r="J36" s="25">
+      <c r="J36" s="22">
         <v>1.02656835</v>
       </c>
-      <c r="K36" s="24"/>
+      <c r="K36" s="21"/>
       <c r="L36" s="13">
         <v>0</v>
       </c>
@@ -2989,11 +2869,11 @@
       <c r="O36" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="P36" s="25">
+      <c r="P36" s="22">
         <v>671.45</v>
       </c>
-      <c r="Q36" s="24"/>
-      <c r="R36" s="24"/>
+      <c r="Q36" s="21"/>
+      <c r="R36" s="21"/>
       <c r="S36" s="3" t="s">
         <v>35</v>
       </c>
@@ -3006,7 +2886,7 @@
       <c r="V36" s="13">
         <v>0</v>
       </c>
-      <c r="W36" s="27"/>
+      <c r="W36" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added a legend that described which plotted box with its id corresponds to which dimensions
</commit_message>
<xml_diff>
--- a/sample_instances/input_small.xlsx
+++ b/sample_instances/input_small.xlsx
@@ -1675,7 +1675,7 @@
         <v>167</v>
       </c>
       <c r="Q14" s="7">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R14" s="15">
         <v>15</v>
@@ -1742,7 +1742,7 @@
         <v>103.37</v>
       </c>
       <c r="Q15" s="7">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R15" s="15">
         <v>5</v>

</xml_diff>